<commit_message>
Polish Synth portfolio presentation
</commit_message>
<xml_diff>
--- a/reports/exports/dataroom-summary.xlsx
+++ b/reports/exports/dataroom-summary.xlsx
@@ -431,7 +431,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>iss-2026-05-12T17-27-46-001</v>
+        <v>iss-2026-05-18T13-26-44-001</v>
       </c>
       <c r="B2" t="str">
         <v>Unilateral Modification Rights</v>
@@ -452,12 +452,12 @@
         <v>Request a mutual written amendment requirement.</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>iss-2026-05-12T17-27-46-002</v>
+        <v>iss-2026-05-18T13-26-44-002</v>
       </c>
       <c r="B3" t="str">
         <v>Limited Liability Cap</v>
@@ -478,12 +478,12 @@
         <v>Negotiate a higher cap and carve-outs for willful misconduct.</v>
       </c>
       <c r="H3" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>iss-2026-05-12T17-27-46-006</v>
+        <v>iss-2026-05-18T13-26-44-006</v>
       </c>
       <c r="B4" t="str">
         <v>Unilateral Modification Rights</v>
@@ -504,12 +504,12 @@
         <v>Request a mutual written amendment requirement.</v>
       </c>
       <c r="H4" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>iss-2026-05-12T17-27-46-007</v>
+        <v>iss-2026-05-18T13-26-44-007</v>
       </c>
       <c r="B5" t="str">
         <v>Limited Liability Cap</v>
@@ -530,12 +530,12 @@
         <v>Negotiate a higher cap and carve-outs for willful misconduct.</v>
       </c>
       <c r="H5" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>iss-2026-05-12T17-27-46-011</v>
+        <v>iss-2026-05-18T13-26-44-011</v>
       </c>
       <c r="B6" t="str">
         <v>Unilateral Modification Rights</v>
@@ -556,12 +556,12 @@
         <v>Request a mutual written amendment requirement.</v>
       </c>
       <c r="H6" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>iss-2026-05-12T17-27-46-012</v>
+        <v>iss-2026-05-18T13-26-44-012</v>
       </c>
       <c r="B7" t="str">
         <v>Limited Liability Cap</v>
@@ -582,12 +582,12 @@
         <v>Negotiate a higher cap and carve-outs for willful misconduct.</v>
       </c>
       <c r="H7" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>iss-2026-05-12T17-27-46-016</v>
+        <v>iss-2026-05-18T13-26-44-016</v>
       </c>
       <c r="B8" t="str">
         <v>Overdue Payments Detected</v>
@@ -608,12 +608,12 @@
         <v>Review overdue invoices against contract payment terms and resolve outstanding amounts.</v>
       </c>
       <c r="H8" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>iss-2026-05-12T17-27-46-017</v>
+        <v>iss-2026-05-18T13-26-44-017</v>
       </c>
       <c r="B9" t="str">
         <v>Overdue Payments Detected</v>
@@ -634,12 +634,12 @@
         <v>Review overdue invoices against contract payment terms and resolve outstanding amounts.</v>
       </c>
       <c r="H9" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>iss-2026-05-12T17-27-46-018</v>
+        <v>iss-2026-05-18T13-26-44-018</v>
       </c>
       <c r="B10" t="str">
         <v>Overdue Payment: DataStream Inc ($9100.00)</v>
@@ -660,12 +660,12 @@
         <v>Resolve overdue payment of $9100.00 to DataStream Inc. Due: 2024-03-31.</v>
       </c>
       <c r="H10" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>iss-2026-05-12T17-27-46-003</v>
+        <v>iss-2026-05-18T13-26-44-003</v>
       </c>
       <c r="B11" t="str">
         <v>Auto-Renewal with Short Notice</v>
@@ -686,12 +686,12 @@
         <v>Calendar the cancellation deadline immediately.</v>
       </c>
       <c r="H11" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>iss-2026-05-12T17-27-46-008</v>
+        <v>iss-2026-05-18T13-26-44-008</v>
       </c>
       <c r="B12" t="str">
         <v>Auto-Renewal with Short Notice</v>
@@ -712,12 +712,12 @@
         <v>Calendar the cancellation deadline immediately.</v>
       </c>
       <c r="H12" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>iss-2026-05-12T17-27-46-013</v>
+        <v>iss-2026-05-18T13-26-44-013</v>
       </c>
       <c r="B13" t="str">
         <v>Auto-Renewal with Short Notice</v>
@@ -738,12 +738,12 @@
         <v>Calendar the cancellation deadline immediately.</v>
       </c>
       <c r="H13" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>iss-2026-05-12T17-27-46-004</v>
+        <v>iss-2026-05-18T13-26-44-004</v>
       </c>
       <c r="B14" t="str">
         <v>Unusual Clause: Unilateral modification rights may allow changes without consent</v>
@@ -764,12 +764,12 @@
         <v>Review this clause with legal counsel to assess acceptability.</v>
       </c>
       <c r="H14" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>iss-2026-05-12T17-27-46-005</v>
+        <v>iss-2026-05-18T13-26-44-005</v>
       </c>
       <c r="B15" t="str">
         <v>Unusual Clause: Review auto-renewal notice window carefully</v>
@@ -790,12 +790,12 @@
         <v>Review this clause with legal counsel to assess acceptability.</v>
       </c>
       <c r="H15" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>iss-2026-05-12T17-27-46-009</v>
+        <v>iss-2026-05-18T13-26-44-009</v>
       </c>
       <c r="B16" t="str">
         <v>Unusual Clause: Unilateral modification rights may allow changes without consent</v>
@@ -816,12 +816,12 @@
         <v>Review this clause with legal counsel to assess acceptability.</v>
       </c>
       <c r="H16" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>iss-2026-05-12T17-27-46-010</v>
+        <v>iss-2026-05-18T13-26-44-010</v>
       </c>
       <c r="B17" t="str">
         <v>Unusual Clause: Review auto-renewal notice window carefully</v>
@@ -842,12 +842,12 @@
         <v>Review this clause with legal counsel to assess acceptability.</v>
       </c>
       <c r="H17" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>iss-2026-05-12T17-27-46-014</v>
+        <v>iss-2026-05-18T13-26-44-014</v>
       </c>
       <c r="B18" t="str">
         <v>Unusual Clause: Unilateral modification rights may allow changes without consent</v>
@@ -868,12 +868,12 @@
         <v>Review this clause with legal counsel to assess acceptability.</v>
       </c>
       <c r="H18" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>iss-2026-05-12T17-27-46-015</v>
+        <v>iss-2026-05-18T13-26-44-015</v>
       </c>
       <c r="B19" t="str">
         <v>Unusual Clause: Review auto-renewal notice window carefully</v>
@@ -894,12 +894,12 @@
         <v>Review this clause with legal counsel to assess acceptability.</v>
       </c>
       <c r="H19" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>iss-2026-05-12T17-27-46-019</v>
+        <v>iss-2026-05-18T13-26-44-019</v>
       </c>
       <c r="B20" t="str">
         <v>Data Quality: High blank cell rate: 40% of cells are empty</v>
@@ -920,12 +920,12 @@
         <v>Review spreadsheet data for completeness and accuracy.</v>
       </c>
       <c r="H20" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>iss-2026-05-12T17-27-46-020</v>
+        <v>iss-2026-05-18T13-26-44-020</v>
       </c>
       <c r="B21" t="str">
         <v>Data Quality: 1 row(s) marked as overdue</v>
@@ -946,12 +946,12 @@
         <v>Review spreadsheet data for completeness and accuracy.</v>
       </c>
       <c r="H21" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>iss-2026-05-12T17-27-46-021</v>
+        <v>iss-2026-05-18T13-26-44-021</v>
       </c>
       <c r="B22" t="str">
         <v>Spreadsheet Warning: High blank cell rate: 40% of cells are empty</v>
@@ -972,12 +972,12 @@
         <v>Review spreadsheet for completeness.</v>
       </c>
       <c r="H22" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>iss-2026-05-12T17-27-46-022</v>
+        <v>iss-2026-05-18T13-26-44-022</v>
       </c>
       <c r="B23" t="str">
         <v>Spreadsheet Warning: 1 row(s) marked as overdue</v>
@@ -998,7 +998,7 @@
         <v>Review spreadsheet for completeness.</v>
       </c>
       <c r="H23" t="str">
-        <v>2026-05-12T17:27:46.736Z</v>
+        <v>2026-05-18T13:26:44.834Z</v>
       </c>
     </row>
   </sheetData>
@@ -1046,10 +1046,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ev-2026-05-12T17-27-46-001</v>
+        <v>ev-2026-05-18T13-26-44-001</v>
       </c>
       <c r="B2" t="str">
-        <v>iss-2026-05-12T17-27-46-001</v>
+        <v>iss-2026-05-18T13-26-44-001</v>
       </c>
       <c r="C2" t="str">
         <v>INDEPENDENT CONTRACTOR AGREEMENT</v>
@@ -1078,10 +1078,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ev-2026-05-12T17-27-46-002</v>
+        <v>ev-2026-05-18T13-26-44-002</v>
       </c>
       <c r="B3" t="str">
-        <v>iss-2026-05-12T17-27-46-002</v>
+        <v>iss-2026-05-18T13-26-44-002</v>
       </c>
       <c r="C3" t="str">
         <v>INDEPENDENT CONTRACTOR AGREEMENT</v>
@@ -1110,10 +1110,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ev-2026-05-12T17-27-46-003</v>
+        <v>ev-2026-05-18T13-26-44-003</v>
       </c>
       <c r="B4" t="str">
-        <v>iss-2026-05-12T17-27-46-003</v>
+        <v>iss-2026-05-18T13-26-44-003</v>
       </c>
       <c r="C4" t="str">
         <v>INDEPENDENT CONTRACTOR AGREEMENT</v>
@@ -1142,10 +1142,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ev-2026-05-12T17-27-46-004</v>
+        <v>ev-2026-05-18T13-26-44-004</v>
       </c>
       <c r="B5" t="str">
-        <v>iss-2026-05-12T17-27-46-004</v>
+        <v>iss-2026-05-18T13-26-44-004</v>
       </c>
       <c r="C5" t="str">
         <v>INDEPENDENT CONTRACTOR AGREEMENT</v>
@@ -1174,10 +1174,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ev-2026-05-12T17-27-46-005</v>
+        <v>ev-2026-05-18T13-26-44-005</v>
       </c>
       <c r="B6" t="str">
-        <v>iss-2026-05-12T17-27-46-005</v>
+        <v>iss-2026-05-18T13-26-44-005</v>
       </c>
       <c r="C6" t="str">
         <v>INDEPENDENT CONTRACTOR AGREEMENT</v>
@@ -1206,10 +1206,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ev-2026-05-12T17-27-46-006</v>
+        <v>ev-2026-05-18T13-26-44-006</v>
       </c>
       <c r="B7" t="str">
-        <v>iss-2026-05-12T17-27-46-006</v>
+        <v>iss-2026-05-18T13-26-44-006</v>
       </c>
       <c r="C7" t="str">
         <v>SAAS SUBSCRIPTION AGREEMENT</v>
@@ -1238,10 +1238,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ev-2026-05-12T17-27-46-007</v>
+        <v>ev-2026-05-18T13-26-44-007</v>
       </c>
       <c r="B8" t="str">
-        <v>iss-2026-05-12T17-27-46-007</v>
+        <v>iss-2026-05-18T13-26-44-007</v>
       </c>
       <c r="C8" t="str">
         <v>SAAS SUBSCRIPTION AGREEMENT</v>
@@ -1270,10 +1270,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ev-2026-05-12T17-27-46-008</v>
+        <v>ev-2026-05-18T13-26-44-008</v>
       </c>
       <c r="B9" t="str">
-        <v>iss-2026-05-12T17-27-46-008</v>
+        <v>iss-2026-05-18T13-26-44-008</v>
       </c>
       <c r="C9" t="str">
         <v>SAAS SUBSCRIPTION AGREEMENT</v>
@@ -1302,10 +1302,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ev-2026-05-12T17-27-46-009</v>
+        <v>ev-2026-05-18T13-26-44-009</v>
       </c>
       <c r="B10" t="str">
-        <v>iss-2026-05-12T17-27-46-009</v>
+        <v>iss-2026-05-18T13-26-44-009</v>
       </c>
       <c r="C10" t="str">
         <v>SAAS SUBSCRIPTION AGREEMENT</v>
@@ -1334,10 +1334,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ev-2026-05-12T17-27-46-010</v>
+        <v>ev-2026-05-18T13-26-44-010</v>
       </c>
       <c r="B11" t="str">
-        <v>iss-2026-05-12T17-27-46-010</v>
+        <v>iss-2026-05-18T13-26-44-010</v>
       </c>
       <c r="C11" t="str">
         <v>SAAS SUBSCRIPTION AGREEMENT</v>
@@ -1366,10 +1366,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ev-2026-05-12T17-27-46-011</v>
+        <v>ev-2026-05-18T13-26-44-011</v>
       </c>
       <c r="B12" t="str">
-        <v>iss-2026-05-12T17-27-46-011</v>
+        <v>iss-2026-05-18T13-26-44-011</v>
       </c>
       <c r="C12" t="str">
         <v>TERM SHEET FOR SERIES A PREFERRED STOCK FINANCING</v>
@@ -1398,10 +1398,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ev-2026-05-12T17-27-46-012</v>
+        <v>ev-2026-05-18T13-26-44-012</v>
       </c>
       <c r="B13" t="str">
-        <v>iss-2026-05-12T17-27-46-012</v>
+        <v>iss-2026-05-18T13-26-44-012</v>
       </c>
       <c r="C13" t="str">
         <v>TERM SHEET FOR SERIES A PREFERRED STOCK FINANCING</v>
@@ -1430,10 +1430,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ev-2026-05-12T17-27-46-013</v>
+        <v>ev-2026-05-18T13-26-44-013</v>
       </c>
       <c r="B14" t="str">
-        <v>iss-2026-05-12T17-27-46-013</v>
+        <v>iss-2026-05-18T13-26-44-013</v>
       </c>
       <c r="C14" t="str">
         <v>TERM SHEET FOR SERIES A PREFERRED STOCK FINANCING</v>
@@ -1462,10 +1462,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ev-2026-05-12T17-27-46-014</v>
+        <v>ev-2026-05-18T13-26-44-014</v>
       </c>
       <c r="B15" t="str">
-        <v>iss-2026-05-12T17-27-46-014</v>
+        <v>iss-2026-05-18T13-26-44-014</v>
       </c>
       <c r="C15" t="str">
         <v>TERM SHEET FOR SERIES A PREFERRED STOCK FINANCING</v>
@@ -1494,10 +1494,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ev-2026-05-12T17-27-46-015</v>
+        <v>ev-2026-05-18T13-26-44-015</v>
       </c>
       <c r="B16" t="str">
-        <v>iss-2026-05-12T17-27-46-015</v>
+        <v>iss-2026-05-18T13-26-44-015</v>
       </c>
       <c r="C16" t="str">
         <v>TERM SHEET FOR SERIES A PREFERRED STOCK FINANCING</v>
@@ -1526,10 +1526,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ev-2026-05-12T17-27-46-016</v>
+        <v>ev-2026-05-18T13-26-44-016</v>
       </c>
       <c r="B17" t="str">
-        <v>iss-2026-05-12T17-27-46-016</v>
+        <v>iss-2026-05-18T13-26-44-016</v>
       </c>
       <c r="C17" t="str">
         <v>sample-contractor-agreement.txt</v>
@@ -1558,10 +1558,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>ev-2026-05-12T17-27-46-017</v>
+        <v>ev-2026-05-18T13-26-44-017</v>
       </c>
       <c r="B18" t="str">
-        <v>iss-2026-05-12T17-27-46-017</v>
+        <v>iss-2026-05-18T13-26-44-017</v>
       </c>
       <c r="C18" t="str">
         <v>sample-contractor-agreement.txt</v>
@@ -1590,10 +1590,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>ev-2026-05-12T17-27-46-018</v>
+        <v>ev-2026-05-18T13-26-44-018</v>
       </c>
       <c r="B19" t="str">
-        <v>iss-2026-05-12T17-27-46-018</v>
+        <v>iss-2026-05-18T13-26-44-018</v>
       </c>
       <c r="C19" t="str">
         <v>sample-payment-schedule.csv</v>
@@ -1622,10 +1622,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>ev-2026-05-12T17-27-46-019</v>
+        <v>ev-2026-05-18T13-26-44-019</v>
       </c>
       <c r="B20" t="str">
-        <v>iss-2026-05-12T17-27-46-019</v>
+        <v>iss-2026-05-18T13-26-44-019</v>
       </c>
       <c r="C20" t="str">
         <v>sample-contractor-agreement.txt</v>
@@ -1654,10 +1654,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ev-2026-05-12T17-27-46-020</v>
+        <v>ev-2026-05-18T13-26-44-020</v>
       </c>
       <c r="B21" t="str">
-        <v>iss-2026-05-12T17-27-46-020</v>
+        <v>iss-2026-05-18T13-26-44-020</v>
       </c>
       <c r="C21" t="str">
         <v>sample-contractor-agreement.txt</v>
@@ -1686,10 +1686,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ev-2026-05-12T17-27-46-021</v>
+        <v>ev-2026-05-18T13-26-44-021</v>
       </c>
       <c r="B22" t="str">
-        <v>iss-2026-05-12T17-27-46-021</v>
+        <v>iss-2026-05-18T13-26-44-021</v>
       </c>
       <c r="C22" t="str">
         <v>sample-cap-table.csv</v>
@@ -1718,10 +1718,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ev-2026-05-12T17-27-46-022</v>
+        <v>ev-2026-05-18T13-26-44-022</v>
       </c>
       <c r="B23" t="str">
-        <v>iss-2026-05-12T17-27-46-022</v>
+        <v>iss-2026-05-18T13-26-44-022</v>
       </c>
       <c r="C23" t="str">
         <v>sample-payment-schedule.csv</v>
@@ -2262,7 +2262,7 @@
         <v>Generated At</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-05-12T11:20:02.571Z</v>
+        <v>2026-05-18T13:26:42.562Z</v>
       </c>
     </row>
     <row r="4">

</xml_diff>